<commit_message>
module grids get the same pages and a plot index
</commit_message>
<xml_diff>
--- a/04_Network/03_Classify/c_data/03_classify.xlsx
+++ b/04_Network/03_Classify/c_data/03_classify.xlsx
@@ -10,15 +10,16 @@
     <sheet name="read_me" sheetId="1" r:id="rId1"/>
     <sheet name="counts" sheetId="2" r:id="rId2"/>
     <sheet name="auc" sheetId="3" r:id="rId3"/>
-    <sheet name="input_manifest" sheetId="4" r:id="rId4"/>
-    <sheet name="package_versions" sheetId="5" r:id="rId5"/>
+    <sheet name="plot_index" sheetId="4" r:id="rId4"/>
+    <sheet name="input_manifest" sheetId="5" r:id="rId5"/>
+    <sheet name="package_versions" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="551" uniqueCount="124">
   <si>
     <t>sheet</t>
   </si>
@@ -38,6 +39,12 @@
     <t>Per module and task: AUC, median paired change (paired tasks), Wilcoxon p and BH FDR.</t>
   </si>
   <si>
+    <t>plot_index</t>
+  </si>
+  <si>
+    <t>PDF page and panel position (1 to 12) of every p &lt; 0.05 row of auc.</t>
+  </si>
+  <si>
     <t>input_manifest</t>
   </si>
   <si>
@@ -104,7 +111,7 @@
     <t>Baseline_HRvLR</t>
   </si>
   <si>
-    <t>HR vs LR at T1 (floor)</t>
+    <t>HR vs LR at T1</t>
   </si>
   <si>
     <t>Trained_HRvLR</t>
@@ -174,6 +181,12 @@
   </si>
   <si>
     <t>pink</t>
+  </si>
+  <si>
+    <t>pdf_page</t>
+  </si>
+  <si>
+    <t>position</t>
   </si>
   <si>
     <t>input</t>
@@ -720,7 +733,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1">
@@ -761,6 +774,14 @@
       </c>
       <c r="B5" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -775,39 +796,39 @@
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
@@ -833,10 +854,10 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C3" t="b">
         <v>1</v>
@@ -862,10 +883,10 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C4" t="b">
         <v>1</v>
@@ -891,10 +912,10 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C5" t="b">
         <v>1</v>
@@ -920,10 +941,10 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C6" t="b">
         <v>0</v>
@@ -949,10 +970,10 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C7" t="b">
         <v>0</v>
@@ -978,10 +999,10 @@
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C8" t="b">
         <v>0</v>
@@ -1007,10 +1028,10 @@
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C9" t="b">
         <v>0</v>
@@ -1046,54 +1067,54 @@
   <sheetData>
     <row r="1" spans="1:11" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F2">
         <v>0.1836734693877551</v>
@@ -1116,19 +1137,19 @@
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C3" t="b">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F3">
         <v>0.9183673469387755</v>
@@ -1151,19 +1172,19 @@
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C4" t="b">
         <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F4">
         <v>0.2448979591836735</v>
@@ -1186,19 +1207,19 @@
     </row>
     <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C5" t="b">
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F5">
         <v>0.2244897959183673</v>
@@ -1221,19 +1242,19 @@
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C6" t="b">
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F6">
         <v>0.7346938775510204</v>
@@ -1256,19 +1277,19 @@
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C7" t="b">
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E7" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F7">
         <v>0.6938775510204082</v>
@@ -1291,19 +1312,19 @@
     </row>
     <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C8" t="b">
         <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F8">
         <v>0.5714285714285714</v>
@@ -1326,19 +1347,19 @@
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C9" t="b">
         <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F9">
         <v>0.6938775510204082</v>
@@ -1361,19 +1382,19 @@
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C10" t="b">
         <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E10" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F10">
         <v>0.3469387755102041</v>
@@ -1396,19 +1417,19 @@
     </row>
     <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B11" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C11" t="b">
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E11" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F11">
         <v>0.4897959183673469</v>
@@ -1431,19 +1452,19 @@
     </row>
     <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B12" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C12" t="b">
         <v>1</v>
       </c>
       <c r="D12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F12">
         <v>0.6530612244897959</v>
@@ -1466,19 +1487,19 @@
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C13" t="b">
         <v>1</v>
       </c>
       <c r="D13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F13">
         <v>0.5918367346938775</v>
@@ -1501,19 +1522,19 @@
     </row>
     <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B14" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C14" t="b">
         <v>1</v>
       </c>
       <c r="D14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F14">
         <v>0.859375</v>
@@ -1536,19 +1557,19 @@
     </row>
     <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C15" t="b">
         <v>1</v>
       </c>
       <c r="D15" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E15" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F15">
         <v>0.171875</v>
@@ -1571,19 +1592,19 @@
     </row>
     <row r="16" spans="1:11">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C16" t="b">
         <v>1</v>
       </c>
       <c r="D16" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E16" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F16">
         <v>0.78125</v>
@@ -1606,19 +1627,19 @@
     </row>
     <row r="17" spans="1:11">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C17" t="b">
         <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E17" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F17">
         <v>0.265625</v>
@@ -1641,19 +1662,19 @@
     </row>
     <row r="18" spans="1:11">
       <c r="A18" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B18" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C18" t="b">
         <v>1</v>
       </c>
       <c r="D18" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E18" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F18">
         <v>0.765625</v>
@@ -1676,19 +1697,19 @@
     </row>
     <row r="19" spans="1:11">
       <c r="A19" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B19" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C19" t="b">
         <v>1</v>
       </c>
       <c r="D19" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E19" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F19">
         <v>0.671875</v>
@@ -1711,19 +1732,19 @@
     </row>
     <row r="20" spans="1:11">
       <c r="A20" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B20" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C20" t="b">
         <v>1</v>
       </c>
       <c r="D20" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E20" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F20">
         <v>0.390625</v>
@@ -1746,19 +1767,19 @@
     </row>
     <row r="21" spans="1:11">
       <c r="A21" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B21" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C21" t="b">
         <v>1</v>
       </c>
       <c r="D21" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E21" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F21">
         <v>0.34375</v>
@@ -1781,19 +1802,19 @@
     </row>
     <row r="22" spans="1:11">
       <c r="A22" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B22" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C22" t="b">
         <v>1</v>
       </c>
       <c r="D22" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E22" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F22">
         <v>0.609375</v>
@@ -1816,19 +1837,19 @@
     </row>
     <row r="23" spans="1:11">
       <c r="A23" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B23" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C23" t="b">
         <v>1</v>
       </c>
       <c r="D23" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E23" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F23">
         <v>0.5625</v>
@@ -1851,19 +1872,19 @@
     </row>
     <row r="24" spans="1:11">
       <c r="A24" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B24" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C24" t="b">
         <v>1</v>
       </c>
       <c r="D24" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E24" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F24">
         <v>0.609375</v>
@@ -1886,19 +1907,19 @@
     </row>
     <row r="25" spans="1:11">
       <c r="A25" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B25" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C25" t="b">
         <v>1</v>
       </c>
       <c r="D25" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E25" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F25">
         <v>0.390625</v>
@@ -1921,19 +1942,19 @@
     </row>
     <row r="26" spans="1:11">
       <c r="A26" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B26" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C26" t="b">
         <v>0</v>
       </c>
       <c r="D26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F26">
         <v>0.1964285714285714</v>
@@ -1953,19 +1974,19 @@
     </row>
     <row r="27" spans="1:11">
       <c r="A27" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B27" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C27" t="b">
         <v>0</v>
       </c>
       <c r="D27" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E27" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F27">
         <v>0.7857142857142857</v>
@@ -1985,19 +2006,19 @@
     </row>
     <row r="28" spans="1:11">
       <c r="A28" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B28" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C28" t="b">
         <v>0</v>
       </c>
       <c r="D28" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E28" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F28">
         <v>0.2321428571428572</v>
@@ -2017,19 +2038,19 @@
     </row>
     <row r="29" spans="1:11">
       <c r="A29" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B29" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C29" t="b">
         <v>0</v>
       </c>
       <c r="D29" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E29" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F29">
         <v>0.7321428571428571</v>
@@ -2049,19 +2070,19 @@
     </row>
     <row r="30" spans="1:11">
       <c r="A30" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B30" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C30" t="b">
         <v>0</v>
       </c>
       <c r="D30" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E30" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F30">
         <v>0.3035714285714285</v>
@@ -2081,19 +2102,19 @@
     </row>
     <row r="31" spans="1:11">
       <c r="A31" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B31" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C31" t="b">
         <v>0</v>
       </c>
       <c r="D31" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E31" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F31">
         <v>0.3392857142857143</v>
@@ -2113,19 +2134,19 @@
     </row>
     <row r="32" spans="1:11">
       <c r="A32" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B32" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C32" t="b">
         <v>0</v>
       </c>
       <c r="D32" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E32" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F32">
         <v>0.6607142857142857</v>
@@ -2145,19 +2166,19 @@
     </row>
     <row r="33" spans="1:11">
       <c r="A33" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B33" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C33" t="b">
         <v>0</v>
       </c>
       <c r="D33" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E33" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F33">
         <v>0.4107142857142857</v>
@@ -2177,19 +2198,19 @@
     </row>
     <row r="34" spans="1:11">
       <c r="A34" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B34" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C34" t="b">
         <v>0</v>
       </c>
       <c r="D34" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E34" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F34">
         <v>0.5357142857142857</v>
@@ -2209,19 +2230,19 @@
     </row>
     <row r="35" spans="1:11">
       <c r="A35" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B35" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C35" t="b">
         <v>0</v>
       </c>
       <c r="D35" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E35" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F35">
         <v>0.5178571428571429</v>
@@ -2241,19 +2262,19 @@
     </row>
     <row r="36" spans="1:11">
       <c r="A36" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C36" t="b">
         <v>0</v>
       </c>
       <c r="D36" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E36" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F36">
         <v>0.4821428571428572</v>
@@ -2273,19 +2294,19 @@
     </row>
     <row r="37" spans="1:11">
       <c r="A37" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C37" t="b">
         <v>0</v>
       </c>
       <c r="D37" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E37" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F37">
         <v>0.4821428571428572</v>
@@ -2305,19 +2326,19 @@
     </row>
     <row r="38" spans="1:11">
       <c r="A38" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B38" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C38" t="b">
         <v>0</v>
       </c>
       <c r="D38" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E38" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F38">
         <v>0.2857142857142857</v>
@@ -2337,19 +2358,19 @@
     </row>
     <row r="39" spans="1:11">
       <c r="A39" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B39" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C39" t="b">
         <v>0</v>
       </c>
       <c r="D39" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E39" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F39">
         <v>0.7142857142857143</v>
@@ -2369,19 +2390,19 @@
     </row>
     <row r="40" spans="1:11">
       <c r="A40" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B40" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C40" t="b">
         <v>0</v>
       </c>
       <c r="D40" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E40" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F40">
         <v>0.3214285714285715</v>
@@ -2401,19 +2422,19 @@
     </row>
     <row r="41" spans="1:11">
       <c r="A41" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B41" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C41" t="b">
         <v>0</v>
       </c>
       <c r="D41" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E41" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F41">
         <v>0.6607142857142857</v>
@@ -2433,19 +2454,19 @@
     </row>
     <row r="42" spans="1:11">
       <c r="A42" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B42" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C42" t="b">
         <v>0</v>
       </c>
       <c r="D42" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E42" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F42">
         <v>0.625</v>
@@ -2465,19 +2486,19 @@
     </row>
     <row r="43" spans="1:11">
       <c r="A43" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B43" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C43" t="b">
         <v>0</v>
       </c>
       <c r="D43" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E43" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F43">
         <v>0.4464285714285715</v>
@@ -2497,19 +2518,19 @@
     </row>
     <row r="44" spans="1:11">
       <c r="A44" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B44" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C44" t="b">
         <v>0</v>
       </c>
       <c r="D44" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E44" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F44">
         <v>0.5535714285714286</v>
@@ -2529,19 +2550,19 @@
     </row>
     <row r="45" spans="1:11">
       <c r="A45" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B45" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C45" t="b">
         <v>0</v>
       </c>
       <c r="D45" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E45" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F45">
         <v>0.5357142857142857</v>
@@ -2561,19 +2582,19 @@
     </row>
     <row r="46" spans="1:11">
       <c r="A46" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B46" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C46" t="b">
         <v>0</v>
       </c>
       <c r="D46" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E46" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F46">
         <v>0.5357142857142857</v>
@@ -2593,19 +2614,19 @@
     </row>
     <row r="47" spans="1:11">
       <c r="A47" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B47" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C47" t="b">
         <v>0</v>
       </c>
       <c r="D47" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E47" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F47">
         <v>0.5357142857142857</v>
@@ -2625,19 +2646,19 @@
     </row>
     <row r="48" spans="1:11">
       <c r="A48" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B48" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C48" t="b">
         <v>0</v>
       </c>
       <c r="D48" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E48" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F48">
         <v>0.5178571428571429</v>
@@ -2657,19 +2678,19 @@
     </row>
     <row r="49" spans="1:11">
       <c r="A49" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B49" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C49" t="b">
         <v>0</v>
       </c>
       <c r="D49" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E49" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F49">
         <v>0.5</v>
@@ -2689,19 +2710,19 @@
     </row>
     <row r="50" spans="1:11">
       <c r="A50" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B50" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C50" t="b">
         <v>0</v>
       </c>
       <c r="D50" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E50" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F50">
         <v>0.7678571428571429</v>
@@ -2721,19 +2742,19 @@
     </row>
     <row r="51" spans="1:11">
       <c r="A51" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B51" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C51" t="b">
         <v>0</v>
       </c>
       <c r="D51" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E51" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F51">
         <v>0.7321428571428571</v>
@@ -2753,19 +2774,19 @@
     </row>
     <row r="52" spans="1:11">
       <c r="A52" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B52" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C52" t="b">
         <v>0</v>
       </c>
       <c r="D52" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E52" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F52">
         <v>0.7142857142857143</v>
@@ -2785,19 +2806,19 @@
     </row>
     <row r="53" spans="1:11">
       <c r="A53" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B53" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C53" t="b">
         <v>0</v>
       </c>
       <c r="D53" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E53" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F53">
         <v>0.6964285714285714</v>
@@ -2817,19 +2838,19 @@
     </row>
     <row r="54" spans="1:11">
       <c r="A54" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B54" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C54" t="b">
         <v>0</v>
       </c>
       <c r="D54" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E54" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F54">
         <v>0.3035714285714285</v>
@@ -2849,19 +2870,19 @@
     </row>
     <row r="55" spans="1:11">
       <c r="A55" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B55" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C55" t="b">
         <v>0</v>
       </c>
       <c r="D55" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E55" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F55">
         <v>0.3571428571428572</v>
@@ -2881,19 +2902,19 @@
     </row>
     <row r="56" spans="1:11">
       <c r="A56" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B56" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C56" t="b">
         <v>0</v>
       </c>
       <c r="D56" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E56" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F56">
         <v>0.375</v>
@@ -2913,19 +2934,19 @@
     </row>
     <row r="57" spans="1:11">
       <c r="A57" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B57" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C57" t="b">
         <v>0</v>
       </c>
       <c r="D57" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E57" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F57">
         <v>0.6071428571428571</v>
@@ -2945,19 +2966,19 @@
     </row>
     <row r="58" spans="1:11">
       <c r="A58" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B58" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C58" t="b">
         <v>0</v>
       </c>
       <c r="D58" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E58" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F58">
         <v>0.4107142857142857</v>
@@ -2977,19 +2998,19 @@
     </row>
     <row r="59" spans="1:11">
       <c r="A59" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B59" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C59" t="b">
         <v>0</v>
       </c>
       <c r="D59" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E59" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F59">
         <v>0.4285714285714285</v>
@@ -3009,19 +3030,19 @@
     </row>
     <row r="60" spans="1:11">
       <c r="A60" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B60" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C60" t="b">
         <v>0</v>
       </c>
       <c r="D60" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E60" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F60">
         <v>0.4285714285714285</v>
@@ -3041,19 +3062,19 @@
     </row>
     <row r="61" spans="1:11">
       <c r="A61" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B61" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C61" t="b">
         <v>0</v>
       </c>
       <c r="D61" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E61" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F61">
         <v>0.4464285714285715</v>
@@ -3073,19 +3094,19 @@
     </row>
     <row r="62" spans="1:11">
       <c r="A62" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B62" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C62" t="b">
         <v>1</v>
       </c>
       <c r="D62" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E62" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F62">
         <v>0.8888888888888888</v>
@@ -3108,19 +3129,19 @@
     </row>
     <row r="63" spans="1:11">
       <c r="A63" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B63" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C63" t="b">
         <v>1</v>
       </c>
       <c r="D63" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E63" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F63">
         <v>0.3055555555555556</v>
@@ -3143,19 +3164,19 @@
     </row>
     <row r="64" spans="1:11">
       <c r="A64" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B64" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C64" t="b">
         <v>1</v>
       </c>
       <c r="D64" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E64" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F64">
         <v>0.6944444444444444</v>
@@ -3178,19 +3199,19 @@
     </row>
     <row r="65" spans="1:11">
       <c r="A65" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B65" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C65" t="b">
         <v>1</v>
       </c>
       <c r="D65" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E65" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F65">
         <v>0.6388888888888888</v>
@@ -3213,19 +3234,19 @@
     </row>
     <row r="66" spans="1:11">
       <c r="A66" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B66" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C66" t="b">
         <v>1</v>
       </c>
       <c r="D66" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E66" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F66">
         <v>0.1388888888888889</v>
@@ -3248,19 +3269,19 @@
     </row>
     <row r="67" spans="1:11">
       <c r="A67" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B67" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C67" t="b">
         <v>1</v>
       </c>
       <c r="D67" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E67" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F67">
         <v>0.6666666666666666</v>
@@ -3283,19 +3304,19 @@
     </row>
     <row r="68" spans="1:11">
       <c r="A68" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B68" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C68" t="b">
         <v>1</v>
       </c>
       <c r="D68" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E68" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F68">
         <v>0.5277777777777778</v>
@@ -3318,19 +3339,19 @@
     </row>
     <row r="69" spans="1:11">
       <c r="A69" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B69" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C69" t="b">
         <v>1</v>
       </c>
       <c r="D69" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E69" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F69">
         <v>0.5</v>
@@ -3353,19 +3374,19 @@
     </row>
     <row r="70" spans="1:11">
       <c r="A70" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B70" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C70" t="b">
         <v>1</v>
       </c>
       <c r="D70" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E70" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F70">
         <v>0.4166666666666667</v>
@@ -3388,19 +3409,19 @@
     </row>
     <row r="71" spans="1:11">
       <c r="A71" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B71" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C71" t="b">
         <v>1</v>
       </c>
       <c r="D71" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E71" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F71">
         <v>0.5277777777777778</v>
@@ -3423,19 +3444,19 @@
     </row>
     <row r="72" spans="1:11">
       <c r="A72" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B72" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C72" t="b">
         <v>1</v>
       </c>
       <c r="D72" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E72" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F72">
         <v>0.6111111111111112</v>
@@ -3458,19 +3479,19 @@
     </row>
     <row r="73" spans="1:11">
       <c r="A73" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B73" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C73" t="b">
         <v>1</v>
       </c>
       <c r="D73" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E73" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F73">
         <v>0.4722222222222222</v>
@@ -3493,19 +3514,19 @@
     </row>
     <row r="74" spans="1:11">
       <c r="A74" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B74" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C74" t="b">
         <v>1</v>
       </c>
       <c r="D74" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E74" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F74">
         <v>0.6875</v>
@@ -3528,19 +3549,19 @@
     </row>
     <row r="75" spans="1:11">
       <c r="A75" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B75" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C75" t="b">
         <v>1</v>
       </c>
       <c r="D75" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E75" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F75">
         <v>0.515625</v>
@@ -3563,19 +3584,19 @@
     </row>
     <row r="76" spans="1:11">
       <c r="A76" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B76" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C76" t="b">
         <v>1</v>
       </c>
       <c r="D76" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E76" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F76">
         <v>0.421875</v>
@@ -3598,19 +3619,19 @@
     </row>
     <row r="77" spans="1:11">
       <c r="A77" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B77" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C77" t="b">
         <v>1</v>
       </c>
       <c r="D77" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E77" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F77">
         <v>0.578125</v>
@@ -3633,19 +3654,19 @@
     </row>
     <row r="78" spans="1:11">
       <c r="A78" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B78" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C78" t="b">
         <v>1</v>
       </c>
       <c r="D78" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E78" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F78">
         <v>0.40625</v>
@@ -3668,19 +3689,19 @@
     </row>
     <row r="79" spans="1:11">
       <c r="A79" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B79" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C79" t="b">
         <v>1</v>
       </c>
       <c r="D79" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E79" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F79">
         <v>0.46875</v>
@@ -3703,19 +3724,19 @@
     </row>
     <row r="80" spans="1:11">
       <c r="A80" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B80" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C80" t="b">
         <v>1</v>
       </c>
       <c r="D80" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E80" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F80">
         <v>0.515625</v>
@@ -3738,19 +3759,19 @@
     </row>
     <row r="81" spans="1:11">
       <c r="A81" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B81" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C81" t="b">
         <v>1</v>
       </c>
       <c r="D81" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E81" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F81">
         <v>0.5</v>
@@ -3773,19 +3794,19 @@
     </row>
     <row r="82" spans="1:11">
       <c r="A82" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B82" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C82" t="b">
         <v>1</v>
       </c>
       <c r="D82" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E82" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F82">
         <v>0.4375</v>
@@ -3808,19 +3829,19 @@
     </row>
     <row r="83" spans="1:11">
       <c r="A83" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B83" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C83" t="b">
         <v>1</v>
       </c>
       <c r="D83" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E83" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F83">
         <v>0.390625</v>
@@ -3843,19 +3864,19 @@
     </row>
     <row r="84" spans="1:11">
       <c r="A84" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B84" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C84" t="b">
         <v>1</v>
       </c>
       <c r="D84" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E84" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F84">
         <v>0.46875</v>
@@ -3878,19 +3899,19 @@
     </row>
     <row r="85" spans="1:11">
       <c r="A85" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B85" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C85" t="b">
         <v>1</v>
       </c>
       <c r="D85" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E85" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F85">
         <v>0.625</v>
@@ -3913,19 +3934,19 @@
     </row>
     <row r="86" spans="1:11">
       <c r="A86" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B86" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C86" t="b">
         <v>0</v>
       </c>
       <c r="D86" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E86" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F86">
         <v>0.7291666666666666</v>
@@ -3945,19 +3966,19 @@
     </row>
     <row r="87" spans="1:11">
       <c r="A87" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B87" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C87" t="b">
         <v>0</v>
       </c>
       <c r="D87" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E87" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F87">
         <v>0.6666666666666666</v>
@@ -3977,19 +3998,19 @@
     </row>
     <row r="88" spans="1:11">
       <c r="A88" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B88" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C88" t="b">
         <v>0</v>
       </c>
       <c r="D88" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E88" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F88">
         <v>0.3333333333333333</v>
@@ -4009,19 +4030,19 @@
     </row>
     <row r="89" spans="1:11">
       <c r="A89" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B89" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C89" t="b">
         <v>0</v>
       </c>
       <c r="D89" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E89" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F89">
         <v>0.3541666666666667</v>
@@ -4041,19 +4062,19 @@
     </row>
     <row r="90" spans="1:11">
       <c r="A90" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B90" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C90" t="b">
         <v>0</v>
       </c>
       <c r="D90" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E90" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F90">
         <v>0.625</v>
@@ -4073,19 +4094,19 @@
     </row>
     <row r="91" spans="1:11">
       <c r="A91" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B91" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C91" t="b">
         <v>0</v>
       </c>
       <c r="D91" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E91" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F91">
         <v>0.6041666666666666</v>
@@ -4105,19 +4126,19 @@
     </row>
     <row r="92" spans="1:11">
       <c r="A92" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B92" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C92" t="b">
         <v>0</v>
       </c>
       <c r="D92" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E92" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F92">
         <v>0.4375</v>
@@ -4137,19 +4158,19 @@
     </row>
     <row r="93" spans="1:11">
       <c r="A93" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B93" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C93" t="b">
         <v>0</v>
       </c>
       <c r="D93" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E93" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F93">
         <v>0.4583333333333333</v>
@@ -4169,19 +4190,19 @@
     </row>
     <row r="94" spans="1:11">
       <c r="A94" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B94" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C94" t="b">
         <v>0</v>
       </c>
       <c r="D94" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E94" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F94">
         <v>0.5416666666666666</v>
@@ -4201,19 +4222,19 @@
     </row>
     <row r="95" spans="1:11">
       <c r="A95" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B95" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C95" t="b">
         <v>0</v>
       </c>
       <c r="D95" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E95" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F95">
         <v>0.4791666666666667</v>
@@ -4233,19 +4254,19 @@
     </row>
     <row r="96" spans="1:11">
       <c r="A96" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B96" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C96" t="b">
         <v>0</v>
       </c>
       <c r="D96" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E96" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F96">
         <v>0.5</v>
@@ -4265,19 +4286,19 @@
     </row>
     <row r="97" spans="1:11">
       <c r="A97" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B97" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C97" t="b">
         <v>0</v>
       </c>
       <c r="D97" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E97" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F97">
         <v>0.5</v>
@@ -4302,29 +4323,126 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1">
+    <row r="1" spans="1:5" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>52</v>
+        <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="E1" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="C2" t="s">
-        <v>57</v>
+        <v>44</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -4334,337 +4452,369 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4" t="s">
         <v>67</v>
-      </c>
-      <c r="C4" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B5" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C5" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B6" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C6" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B7" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C7" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B8" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C8" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B9" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C9" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B10" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C10" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B11" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C11" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B12" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C12" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B13" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C13" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B14" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C14" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B15" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C15" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B16" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C16" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B17" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C17" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B18" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C18" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B19" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C19" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B20" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C20" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B21" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C21" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B22" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C22" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B23" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C23" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B24" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C24" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B25" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C25" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B26" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C26" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B27" t="s">
+        <v>71</v>
+      </c>
+      <c r="C27" t="s">
         <v>67</v>
-      </c>
-      <c r="C27" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B28" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C28" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B29" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C29" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B30" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C30" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
classify scripts share one heatmap, grid and workbook block
</commit_message>
<xml_diff>
--- a/04_Network/03_Classify/c_data/03_classify.xlsx
+++ b/04_Network/03_Classify/c_data/03_classify.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="170">
   <si>
     <t>sheet</t>
   </si>
@@ -192,16 +192,19 @@
     <t>overview</t>
   </si>
   <si>
+    <t>Classification overview: modules</t>
+  </si>
+  <si>
+    <t>input</t>
+  </si>
+  <si>
+    <t>path</t>
+  </si>
+  <si>
+    <t>md5</t>
+  </si>
+  <si>
     <t>modules</t>
-  </si>
-  <si>
-    <t>input</t>
-  </si>
-  <si>
-    <t>path</t>
-  </si>
-  <si>
-    <t>md5</t>
   </si>
   <si>
     <t>04_Network/01_Build_Modules/c_data/modules.rds</t>
@@ -4614,13 +4617,13 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -4635,574 +4638,574 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C4" t="s">
         <v>72</v>
-      </c>
-      <c r="B4" t="s">
-        <v>73</v>
-      </c>
-      <c r="C4" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C10" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B13" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B15" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B16" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C16" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B17" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C17" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C18" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B19" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C19" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B20" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C20" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B21" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C21" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B22" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C22" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B23" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C23" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B24" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C24" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B25" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C25" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B26" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C26" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B27" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C27" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B28" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C28" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B29" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C29" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B30" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C30" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B31" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C31" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B32" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C32" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C33" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B34" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C34" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B35" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C35" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B36" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C36" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C37" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B38" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C38" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B39" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C39" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B40" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C40" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B41" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C41" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B42" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C42" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B43" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C43" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B44" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C44" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B45" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C45" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B46" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C46" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B47" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C47" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B48" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C48" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B49" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C49" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B50" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C50" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B51" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C51" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B52" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C52" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
rerun on the q-value scripts; only new columns and the hit text change
</commit_message>
<xml_diff>
--- a/04_Network/03_Classify/c_data/03_classify.xlsx
+++ b/04_Network/03_Classify/c_data/03_classify.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="741" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="742" uniqueCount="180">
   <si>
     <t>sheet</t>
   </si>
@@ -36,7 +36,7 @@
     <t>auc</t>
   </si>
   <si>
-    <t>Per module and task: AUC, median paired change (paired tasks), Wilcoxon p and BH FDR.</t>
+    <t>Per module and task: AUC, median paired change (paired tasks), Wilcoxon p, BH and Storey q.</t>
   </si>
   <si>
     <t>plot_index</t>
@@ -151,6 +151,9 @@
   </si>
   <si>
     <t>fdr</t>
+  </si>
+  <si>
+    <t>qvalue</t>
   </si>
   <si>
     <t>blue</t>
@@ -1227,10 +1230,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M121"/>
+  <dimension ref="A1:N121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1">
+    <row r="1" spans="1:14" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -1270,8 +1273,11 @@
       <c r="M1" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="2" spans="1:13">
+      <c r="N1" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
         <v>25</v>
       </c>
@@ -1282,10 +1288,10 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F2">
         <v>0.163265306122449</v>
@@ -1305,8 +1311,11 @@
       <c r="M2">
         <v>0.2343750000000001</v>
       </c>
-    </row>
-    <row r="3" spans="1:13">
+      <c r="N2">
+        <v>0.2343750000000001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -1317,10 +1326,10 @@
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F3">
         <v>0.9183673469387755</v>
@@ -1340,8 +1349,11 @@
       <c r="M3">
         <v>0.2343750000000001</v>
       </c>
-    </row>
-    <row r="4" spans="1:13">
+      <c r="N3">
+        <v>0.2343750000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -1352,10 +1364,10 @@
         <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F4">
         <v>0.6122448979591837</v>
@@ -1375,8 +1387,11 @@
       <c r="M4">
         <v>0.2343750000000001</v>
       </c>
-    </row>
-    <row r="5" spans="1:13">
+      <c r="N4">
+        <v>0.2343750000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -1387,10 +1402,10 @@
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F5">
         <v>0.7755102040816326</v>
@@ -1410,8 +1425,11 @@
       <c r="M5">
         <v>0.4101562500000001</v>
       </c>
-    </row>
-    <row r="6" spans="1:13">
+      <c r="N5">
+        <v>0.4101562500000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -1422,10 +1440,10 @@
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F6">
         <v>0.2448979591836735</v>
@@ -1445,8 +1463,11 @@
       <c r="M6">
         <v>0.4687500000000001</v>
       </c>
-    </row>
-    <row r="7" spans="1:13">
+      <c r="N6">
+        <v>0.4687500000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -1457,10 +1478,10 @@
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F7">
         <v>0.6530612244897959</v>
@@ -1480,8 +1501,11 @@
       <c r="M7">
         <v>0.4687500000000001</v>
       </c>
-    </row>
-    <row r="8" spans="1:13">
+      <c r="N7">
+        <v>0.4687500000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -1492,10 +1516,10 @@
         <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F8">
         <v>0.2040816326530612</v>
@@ -1515,8 +1539,11 @@
       <c r="M8">
         <v>0.4687500000000001</v>
       </c>
-    </row>
-    <row r="9" spans="1:13">
+      <c r="N8">
+        <v>0.4687500000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -1527,10 +1554,10 @@
         <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F9">
         <v>0.2448979591836735</v>
@@ -1550,8 +1577,11 @@
       <c r="M9">
         <v>0.5566406250000001</v>
       </c>
-    </row>
-    <row r="10" spans="1:13">
+      <c r="N9">
+        <v>0.5566406250000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -1562,10 +1592,10 @@
         <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F10">
         <v>0.6938775510204082</v>
@@ -1585,8 +1615,11 @@
       <c r="M10">
         <v>0.7883522727272728</v>
       </c>
-    </row>
-    <row r="11" spans="1:13">
+      <c r="N10">
+        <v>0.7883522727272728</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1597,10 +1630,10 @@
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F11">
         <v>0.6326530612244898</v>
@@ -1620,8 +1653,11 @@
       <c r="M11">
         <v>0.7883522727272728</v>
       </c>
-    </row>
-    <row r="12" spans="1:13">
+      <c r="N11">
+        <v>0.7883522727272728</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -1632,10 +1668,10 @@
         <v>1</v>
       </c>
       <c r="D12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F12">
         <v>0.4489795918367347</v>
@@ -1655,8 +1691,11 @@
       <c r="M12">
         <v>0.7883522727272728</v>
       </c>
-    </row>
-    <row r="13" spans="1:13">
+      <c r="N12">
+        <v>0.7883522727272728</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -1667,10 +1706,10 @@
         <v>1</v>
       </c>
       <c r="D13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F13">
         <v>0.4489795918367347</v>
@@ -1690,8 +1729,11 @@
       <c r="M13">
         <v>0.8125000000000001</v>
       </c>
-    </row>
-    <row r="14" spans="1:13">
+      <c r="N13">
+        <v>0.8125000000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -1702,10 +1744,10 @@
         <v>1</v>
       </c>
       <c r="D14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F14">
         <v>0.5102040816326531</v>
@@ -1725,8 +1767,11 @@
       <c r="M14">
         <v>0.8125000000000001</v>
       </c>
-    </row>
-    <row r="15" spans="1:13">
+      <c r="N14">
+        <v>0.8125000000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
       <c r="A15" t="s">
         <v>25</v>
       </c>
@@ -1737,10 +1782,10 @@
         <v>1</v>
       </c>
       <c r="D15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F15">
         <v>0.5714285714285714</v>
@@ -1760,8 +1805,11 @@
       <c r="M15">
         <v>0.8125000000000001</v>
       </c>
-    </row>
-    <row r="16" spans="1:13">
+      <c r="N15">
+        <v>0.8125000000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -1772,10 +1820,10 @@
         <v>1</v>
       </c>
       <c r="D16" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E16" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F16">
         <v>0.5918367346938775</v>
@@ -1795,8 +1843,11 @@
       <c r="M16">
         <v>0.8125000000000001</v>
       </c>
-    </row>
-    <row r="17" spans="1:13">
+      <c r="N16">
+        <v>0.8125000000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14">
       <c r="A17" t="s">
         <v>27</v>
       </c>
@@ -1807,10 +1858,10 @@
         <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E17" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F17">
         <v>0.171875</v>
@@ -1830,8 +1881,11 @@
       <c r="M17">
         <v>0.03906250000000001</v>
       </c>
-    </row>
-    <row r="18" spans="1:13">
+      <c r="N17">
+        <v>0.03906250000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14">
       <c r="A18" t="s">
         <v>27</v>
       </c>
@@ -1842,10 +1896,10 @@
         <v>1</v>
       </c>
       <c r="D18" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E18" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F18">
         <v>0.734375</v>
@@ -1865,8 +1919,11 @@
       <c r="M18">
         <v>0.03906250000000001</v>
       </c>
-    </row>
-    <row r="19" spans="1:13">
+      <c r="N18">
+        <v>0.03906250000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14">
       <c r="A19" t="s">
         <v>27</v>
       </c>
@@ -1877,10 +1934,10 @@
         <v>1</v>
       </c>
       <c r="D19" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E19" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F19">
         <v>0.09375</v>
@@ -1900,8 +1957,11 @@
       <c r="M19">
         <v>0.03906250000000001</v>
       </c>
-    </row>
-    <row r="20" spans="1:13">
+      <c r="N19">
+        <v>0.03906250000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14">
       <c r="A20" t="s">
         <v>27</v>
       </c>
@@ -1912,10 +1972,10 @@
         <v>1</v>
       </c>
       <c r="D20" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E20" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F20">
         <v>0.84375</v>
@@ -1935,8 +1995,11 @@
       <c r="M20">
         <v>0.05859375000000001</v>
       </c>
-    </row>
-    <row r="21" spans="1:13">
+      <c r="N20">
+        <v>0.05859375000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14">
       <c r="A21" t="s">
         <v>27</v>
       </c>
@@ -1947,10 +2010,10 @@
         <v>1</v>
       </c>
       <c r="D21" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E21" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F21">
         <v>0.171875</v>
@@ -1970,8 +2033,11 @@
       <c r="M21">
         <v>0.05859375000000001</v>
       </c>
-    </row>
-    <row r="22" spans="1:13">
+      <c r="N21">
+        <v>0.05859375000000001</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14">
       <c r="A22" t="s">
         <v>27</v>
       </c>
@@ -1982,10 +2048,10 @@
         <v>1</v>
       </c>
       <c r="D22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F22">
         <v>0.671875</v>
@@ -2005,8 +2071,11 @@
       <c r="M22">
         <v>0.05859375000000001</v>
       </c>
-    </row>
-    <row r="23" spans="1:13">
+      <c r="N22">
+        <v>0.05859375000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14">
       <c r="A23" t="s">
         <v>27</v>
       </c>
@@ -2017,10 +2086,10 @@
         <v>1</v>
       </c>
       <c r="D23" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E23" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F23">
         <v>0.78125</v>
@@ -2040,8 +2109,11 @@
       <c r="M23">
         <v>0.1822916666666667</v>
       </c>
-    </row>
-    <row r="24" spans="1:13">
+      <c r="N23">
+        <v>0.1822916666666667</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14">
       <c r="A24" t="s">
         <v>27</v>
       </c>
@@ -2052,10 +2124,10 @@
         <v>1</v>
       </c>
       <c r="D24" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E24" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F24">
         <v>0.734375</v>
@@ -2075,8 +2147,11 @@
       <c r="M24">
         <v>0.1822916666666667</v>
       </c>
-    </row>
-    <row r="25" spans="1:13">
+      <c r="N24">
+        <v>0.1822916666666667</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14">
       <c r="A25" t="s">
         <v>27</v>
       </c>
@@ -2087,10 +2162,10 @@
         <v>1</v>
       </c>
       <c r="D25" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E25" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F25">
         <v>0.125</v>
@@ -2110,8 +2185,11 @@
       <c r="M25">
         <v>0.1822916666666667</v>
       </c>
-    </row>
-    <row r="26" spans="1:13">
+      <c r="N25">
+        <v>0.1822916666666667</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14">
       <c r="A26" t="s">
         <v>27</v>
       </c>
@@ -2122,10 +2200,10 @@
         <v>1</v>
       </c>
       <c r="D26" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E26" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F26">
         <v>0.328125</v>
@@ -2145,8 +2223,11 @@
       <c r="M26">
         <v>0.5742187500000001</v>
       </c>
-    </row>
-    <row r="27" spans="1:13">
+      <c r="N26">
+        <v>0.5742187500000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14">
       <c r="A27" t="s">
         <v>27</v>
       </c>
@@ -2157,10 +2238,10 @@
         <v>1</v>
       </c>
       <c r="D27" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E27" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F27">
         <v>0.625</v>
@@ -2180,8 +2261,11 @@
       <c r="M27">
         <v>0.7457386363636365</v>
       </c>
-    </row>
-    <row r="28" spans="1:13">
+      <c r="N27">
+        <v>0.7457386363636365</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -2192,10 +2276,10 @@
         <v>1</v>
       </c>
       <c r="D28" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E28" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F28">
         <v>0.625</v>
@@ -2215,8 +2299,11 @@
       <c r="M28">
         <v>0.9040178571428572</v>
       </c>
-    </row>
-    <row r="29" spans="1:13">
+      <c r="N28">
+        <v>0.9040178571428572</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -2227,10 +2314,10 @@
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F29">
         <v>0.515625</v>
@@ -2250,8 +2337,11 @@
       <c r="M29">
         <v>0.9040178571428572</v>
       </c>
-    </row>
-    <row r="30" spans="1:13">
+      <c r="N29">
+        <v>0.9040178571428572</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14">
       <c r="A30" t="s">
         <v>27</v>
       </c>
@@ -2262,10 +2352,10 @@
         <v>1</v>
       </c>
       <c r="D30" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E30" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F30">
         <v>0.484375</v>
@@ -2285,8 +2375,11 @@
       <c r="M30">
         <v>0.9040178571428572</v>
       </c>
-    </row>
-    <row r="31" spans="1:13">
+      <c r="N30">
+        <v>0.9040178571428572</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14">
       <c r="A31" t="s">
         <v>27</v>
       </c>
@@ -2297,10 +2390,10 @@
         <v>1</v>
       </c>
       <c r="D31" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E31" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F31">
         <v>0.46875</v>
@@ -2320,8 +2413,11 @@
       <c r="M31">
         <v>0.9453124999999998</v>
       </c>
-    </row>
-    <row r="32" spans="1:13">
+      <c r="N31">
+        <v>0.9453124999999998</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14">
       <c r="A32" t="s">
         <v>35</v>
       </c>
@@ -2332,10 +2428,10 @@
         <v>0</v>
       </c>
       <c r="D32" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E32" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F32">
         <v>0.9464285714285714</v>
@@ -2358,8 +2454,11 @@
       <c r="M32">
         <v>0.03263403263403263</v>
       </c>
-    </row>
-    <row r="33" spans="1:13">
+      <c r="N32">
+        <v>0.03263403263403263</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14">
       <c r="A33" t="s">
         <v>35</v>
       </c>
@@ -2370,10 +2469,10 @@
         <v>0</v>
       </c>
       <c r="D33" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E33" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F33">
         <v>0.8035714285714286</v>
@@ -2396,8 +2495,11 @@
       <c r="M33">
         <v>0.2703962703962704</v>
       </c>
-    </row>
-    <row r="34" spans="1:13">
+      <c r="N33">
+        <v>0.2703962703962704</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14">
       <c r="A34" t="s">
         <v>35</v>
       </c>
@@ -2408,10 +2510,10 @@
         <v>0</v>
       </c>
       <c r="D34" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E34" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F34">
         <v>0.1964285714285714</v>
@@ -2434,8 +2536,11 @@
       <c r="M34">
         <v>0.2703962703962704</v>
       </c>
-    </row>
-    <row r="35" spans="1:13">
+      <c r="N34">
+        <v>0.2703962703962704</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14">
       <c r="A35" t="s">
         <v>35</v>
       </c>
@@ -2446,10 +2551,10 @@
         <v>0</v>
       </c>
       <c r="D35" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E35" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F35">
         <v>0.2321428571428572</v>
@@ -2472,8 +2577,11 @@
       <c r="M35">
         <v>0.351981351981352</v>
       </c>
-    </row>
-    <row r="36" spans="1:13">
+      <c r="N35">
+        <v>0.351981351981352</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14">
       <c r="A36" t="s">
         <v>35</v>
       </c>
@@ -2484,10 +2592,10 @@
         <v>0</v>
       </c>
       <c r="D36" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E36" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F36">
         <v>0.7142857142857143</v>
@@ -2510,8 +2618,11 @@
       <c r="M36">
         <v>0.5678321678321678</v>
       </c>
-    </row>
-    <row r="37" spans="1:13">
+      <c r="N36">
+        <v>0.5678321678321678</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14">
       <c r="A37" t="s">
         <v>35</v>
       </c>
@@ -2522,10 +2633,10 @@
         <v>0</v>
       </c>
       <c r="D37" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E37" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F37">
         <v>0.3571428571428572</v>
@@ -2548,8 +2659,11 @@
       <c r="M37">
         <v>0.6614866614866616</v>
       </c>
-    </row>
-    <row r="38" spans="1:13">
+      <c r="N37">
+        <v>0.6614866614866616</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14">
       <c r="A38" t="s">
         <v>35</v>
       </c>
@@ -2560,10 +2674,10 @@
         <v>0</v>
       </c>
       <c r="D38" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E38" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F38">
         <v>0.3571428571428572</v>
@@ -2586,8 +2700,11 @@
       <c r="M38">
         <v>0.6614866614866616</v>
       </c>
-    </row>
-    <row r="39" spans="1:13">
+      <c r="N38">
+        <v>0.6614866614866616</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14">
       <c r="A39" t="s">
         <v>35</v>
       </c>
@@ -2598,10 +2715,10 @@
         <v>0</v>
       </c>
       <c r="D39" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E39" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F39">
         <v>0.6428571428571429</v>
@@ -2624,8 +2741,11 @@
       <c r="M39">
         <v>0.6614866614866616</v>
       </c>
-    </row>
-    <row r="40" spans="1:13">
+      <c r="N39">
+        <v>0.6614866614866616</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14">
       <c r="A40" t="s">
         <v>35</v>
       </c>
@@ -2636,10 +2756,10 @@
         <v>0</v>
       </c>
       <c r="D40" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E40" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F40">
         <v>0.6428571428571429</v>
@@ -2662,8 +2782,11 @@
       <c r="M40">
         <v>0.6614866614866616</v>
       </c>
-    </row>
-    <row r="41" spans="1:13">
+      <c r="N40">
+        <v>0.6614866614866616</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14">
       <c r="A41" t="s">
         <v>35</v>
       </c>
@@ -2674,10 +2797,10 @@
         <v>0</v>
       </c>
       <c r="D41" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E41" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F41">
         <v>0.4107142857142857</v>
@@ -2700,8 +2823,11 @@
       <c r="M41">
         <v>0.8665112665112666</v>
       </c>
-    </row>
-    <row r="42" spans="1:13">
+      <c r="N41">
+        <v>0.8665112665112666</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14">
       <c r="A42" t="s">
         <v>35</v>
       </c>
@@ -2712,10 +2838,10 @@
         <v>0</v>
       </c>
       <c r="D42" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E42" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F42">
         <v>0.4464285714285715</v>
@@ -2738,8 +2864,11 @@
       <c r="M42">
         <v>0.8665112665112666</v>
       </c>
-    </row>
-    <row r="43" spans="1:13">
+      <c r="N42">
+        <v>0.8665112665112666</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14">
       <c r="A43" t="s">
         <v>35</v>
       </c>
@@ -2750,10 +2879,10 @@
         <v>0</v>
       </c>
       <c r="D43" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E43" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F43">
         <v>0.4464285714285715</v>
@@ -2776,8 +2905,11 @@
       <c r="M43">
         <v>0.8665112665112666</v>
       </c>
-    </row>
-    <row r="44" spans="1:13">
+      <c r="N43">
+        <v>0.8665112665112666</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14">
       <c r="A44" t="s">
         <v>35</v>
       </c>
@@ -2788,10 +2920,10 @@
         <v>0</v>
       </c>
       <c r="D44" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E44" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F44">
         <v>0.4642857142857143</v>
@@ -2814,8 +2946,11 @@
       <c r="M44">
         <v>0.8665112665112666</v>
       </c>
-    </row>
-    <row r="45" spans="1:13">
+      <c r="N44">
+        <v>0.8665112665112666</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14">
       <c r="A45" t="s">
         <v>35</v>
       </c>
@@ -2826,10 +2961,10 @@
         <v>0</v>
       </c>
       <c r="D45" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E45" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F45">
         <v>0.5357142857142857</v>
@@ -2852,8 +2987,11 @@
       <c r="M45">
         <v>0.8665112665112666</v>
       </c>
-    </row>
-    <row r="46" spans="1:13">
+      <c r="N45">
+        <v>0.8665112665112666</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14">
       <c r="A46" t="s">
         <v>35</v>
       </c>
@@ -2864,10 +3002,10 @@
         <v>0</v>
       </c>
       <c r="D46" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E46" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F46">
         <v>0.4642857142857143</v>
@@ -2890,8 +3028,11 @@
       <c r="M46">
         <v>0.8665112665112666</v>
       </c>
-    </row>
-    <row r="47" spans="1:13">
+      <c r="N46">
+        <v>0.8665112665112666</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14">
       <c r="A47" t="s">
         <v>29</v>
       </c>
@@ -2902,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="D47" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E47" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F47">
         <v>0.8571428571428571</v>
@@ -2928,8 +3069,11 @@
       <c r="M47">
         <v>0.3076923076923077</v>
       </c>
-    </row>
-    <row r="48" spans="1:13">
+      <c r="N47">
+        <v>0.3076923076923077</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14">
       <c r="A48" t="s">
         <v>29</v>
       </c>
@@ -2940,10 +3084,10 @@
         <v>0</v>
       </c>
       <c r="D48" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E48" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F48">
         <v>0.7321428571428571</v>
@@ -2966,8 +3110,11 @@
       <c r="M48">
         <v>0.6951048951048951</v>
       </c>
-    </row>
-    <row r="49" spans="1:13">
+      <c r="N48">
+        <v>0.6951048951048951</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14">
       <c r="A49" t="s">
         <v>29</v>
       </c>
@@ -2978,10 +3125,10 @@
         <v>0</v>
       </c>
       <c r="D49" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E49" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F49">
         <v>0.2857142857142857</v>
@@ -3004,8 +3151,11 @@
       <c r="M49">
         <v>0.6951048951048951</v>
       </c>
-    </row>
-    <row r="50" spans="1:13">
+      <c r="N49">
+        <v>0.6951048951048951</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14">
       <c r="A50" t="s">
         <v>29</v>
       </c>
@@ -3016,10 +3166,10 @@
         <v>0</v>
       </c>
       <c r="D50" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E50" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F50">
         <v>0.7142857142857143</v>
@@ -3042,8 +3192,11 @@
       <c r="M50">
         <v>0.6951048951048951</v>
       </c>
-    </row>
-    <row r="51" spans="1:13">
+      <c r="N50">
+        <v>0.6951048951048951</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14">
       <c r="A51" t="s">
         <v>29</v>
       </c>
@@ -3054,10 +3207,10 @@
         <v>0</v>
       </c>
       <c r="D51" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E51" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F51">
         <v>0.6964285714285714</v>
@@ -3080,8 +3233,11 @@
       <c r="M51">
         <v>0.6951048951048951</v>
       </c>
-    </row>
-    <row r="52" spans="1:13">
+      <c r="N51">
+        <v>0.6951048951048951</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14">
       <c r="A52" t="s">
         <v>29</v>
       </c>
@@ -3092,10 +3248,10 @@
         <v>0</v>
       </c>
       <c r="D52" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E52" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F52">
         <v>0.3214285714285715</v>
@@ -3118,8 +3274,11 @@
       <c r="M52">
         <v>0.6951048951048951</v>
       </c>
-    </row>
-    <row r="53" spans="1:13">
+      <c r="N52">
+        <v>0.6951048951048951</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14">
       <c r="A53" t="s">
         <v>29</v>
       </c>
@@ -3130,10 +3289,10 @@
         <v>0</v>
       </c>
       <c r="D53" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E53" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F53">
         <v>0.6428571428571429</v>
@@ -3156,8 +3315,11 @@
       <c r="M53">
         <v>0.6951048951048951</v>
       </c>
-    </row>
-    <row r="54" spans="1:13">
+      <c r="N53">
+        <v>0.6951048951048951</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14">
       <c r="A54" t="s">
         <v>29</v>
       </c>
@@ -3168,10 +3330,10 @@
         <v>0</v>
       </c>
       <c r="D54" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E54" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F54">
         <v>0.3571428571428572</v>
@@ -3194,8 +3356,11 @@
       <c r="M54">
         <v>0.6951048951048951</v>
       </c>
-    </row>
-    <row r="55" spans="1:13">
+      <c r="N54">
+        <v>0.6951048951048951</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14">
       <c r="A55" t="s">
         <v>29</v>
       </c>
@@ -3206,10 +3371,10 @@
         <v>0</v>
       </c>
       <c r="D55" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E55" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F55">
         <v>0.375</v>
@@ -3232,8 +3397,11 @@
       <c r="M55">
         <v>0.6951048951048951</v>
       </c>
-    </row>
-    <row r="56" spans="1:13">
+      <c r="N55">
+        <v>0.6951048951048951</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14">
       <c r="A56" t="s">
         <v>29</v>
       </c>
@@ -3244,10 +3412,10 @@
         <v>0</v>
       </c>
       <c r="D56" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E56" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F56">
         <v>0.625</v>
@@ -3270,8 +3438,11 @@
       <c r="M56">
         <v>0.6951048951048951</v>
       </c>
-    </row>
-    <row r="57" spans="1:13">
+      <c r="N56">
+        <v>0.6951048951048951</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14">
       <c r="A57" t="s">
         <v>29</v>
       </c>
@@ -3282,10 +3453,10 @@
         <v>0</v>
       </c>
       <c r="D57" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E57" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F57">
         <v>0.4464285714285715</v>
@@ -3308,8 +3479,11 @@
       <c r="M57">
         <v>1</v>
       </c>
-    </row>
-    <row r="58" spans="1:13">
+      <c r="N57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14">
       <c r="A58" t="s">
         <v>29</v>
       </c>
@@ -3320,10 +3494,10 @@
         <v>0</v>
       </c>
       <c r="D58" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E58" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F58">
         <v>0.5178571428571429</v>
@@ -3346,8 +3520,11 @@
       <c r="M58">
         <v>1</v>
       </c>
-    </row>
-    <row r="59" spans="1:13">
+      <c r="N58">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14">
       <c r="A59" t="s">
         <v>29</v>
       </c>
@@ -3358,10 +3535,10 @@
         <v>0</v>
       </c>
       <c r="D59" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E59" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F59">
         <v>0.5178571428571429</v>
@@ -3384,8 +3561,11 @@
       <c r="M59">
         <v>1</v>
       </c>
-    </row>
-    <row r="60" spans="1:13">
+      <c r="N59">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14">
       <c r="A60" t="s">
         <v>29</v>
       </c>
@@ -3396,10 +3576,10 @@
         <v>0</v>
       </c>
       <c r="D60" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E60" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F60">
         <v>0.4821428571428572</v>
@@ -3422,8 +3602,11 @@
       <c r="M60">
         <v>1</v>
       </c>
-    </row>
-    <row r="61" spans="1:13">
+      <c r="N60">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14">
       <c r="A61" t="s">
         <v>29</v>
       </c>
@@ -3434,10 +3617,10 @@
         <v>0</v>
       </c>
       <c r="D61" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E61" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F61">
         <v>0.5</v>
@@ -3460,8 +3643,11 @@
       <c r="M61">
         <v>1</v>
       </c>
-    </row>
-    <row r="62" spans="1:13">
+      <c r="N61">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14">
       <c r="A62" t="s">
         <v>31</v>
       </c>
@@ -3472,10 +3658,10 @@
         <v>0</v>
       </c>
       <c r="D62" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E62" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F62">
         <v>0.7857142857142857</v>
@@ -3498,8 +3684,11 @@
       <c r="M62">
         <v>0.7097902097902099</v>
       </c>
-    </row>
-    <row r="63" spans="1:13">
+      <c r="N62">
+        <v>0.7097902097902099</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14">
       <c r="A63" t="s">
         <v>31</v>
       </c>
@@ -3510,10 +3699,10 @@
         <v>0</v>
       </c>
       <c r="D63" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E63" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F63">
         <v>0.75</v>
@@ -3536,8 +3725,11 @@
       <c r="M63">
         <v>0.7097902097902099</v>
       </c>
-    </row>
-    <row r="64" spans="1:13">
+      <c r="N63">
+        <v>0.7097902097902099</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14">
       <c r="A64" t="s">
         <v>31</v>
       </c>
@@ -3548,10 +3740,10 @@
         <v>0</v>
       </c>
       <c r="D64" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E64" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F64">
         <v>0.2678571428571428</v>
@@ -3574,8 +3766,11 @@
       <c r="M64">
         <v>0.7097902097902099</v>
       </c>
-    </row>
-    <row r="65" spans="1:13">
+      <c r="N64">
+        <v>0.7097902097902099</v>
+      </c>
+    </row>
+    <row r="65" spans="1:14">
       <c r="A65" t="s">
         <v>31</v>
       </c>
@@ -3586,10 +3781,10 @@
         <v>0</v>
       </c>
       <c r="D65" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E65" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F65">
         <v>0.2857142857142857</v>
@@ -3612,8 +3807,11 @@
       <c r="M65">
         <v>0.7097902097902099</v>
       </c>
-    </row>
-    <row r="66" spans="1:13">
+      <c r="N65">
+        <v>0.7097902097902099</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14">
       <c r="A66" t="s">
         <v>31</v>
       </c>
@@ -3624,10 +3822,10 @@
         <v>0</v>
       </c>
       <c r="D66" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E66" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F66">
         <v>0.6428571428571429</v>
@@ -3650,8 +3848,11 @@
       <c r="M66">
         <v>0.7441724941724943</v>
       </c>
-    </row>
-    <row r="67" spans="1:13">
+      <c r="N66">
+        <v>0.7441724941724943</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14">
       <c r="A67" t="s">
         <v>31</v>
       </c>
@@ -3662,10 +3863,10 @@
         <v>0</v>
       </c>
       <c r="D67" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E67" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F67">
         <v>0.6428571428571429</v>
@@ -3688,8 +3889,11 @@
       <c r="M67">
         <v>0.7441724941724943</v>
       </c>
-    </row>
-    <row r="68" spans="1:13">
+      <c r="N67">
+        <v>0.7441724941724943</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14">
       <c r="A68" t="s">
         <v>31</v>
       </c>
@@ -3700,10 +3904,10 @@
         <v>0</v>
       </c>
       <c r="D68" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E68" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F68">
         <v>0.6428571428571429</v>
@@ -3726,8 +3930,11 @@
       <c r="M68">
         <v>0.7441724941724943</v>
       </c>
-    </row>
-    <row r="69" spans="1:13">
+      <c r="N68">
+        <v>0.7441724941724943</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14">
       <c r="A69" t="s">
         <v>31</v>
       </c>
@@ -3738,10 +3945,10 @@
         <v>0</v>
       </c>
       <c r="D69" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E69" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F69">
         <v>0.3571428571428572</v>
@@ -3764,8 +3971,11 @@
       <c r="M69">
         <v>0.7441724941724943</v>
       </c>
-    </row>
-    <row r="70" spans="1:13">
+      <c r="N69">
+        <v>0.7441724941724943</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14">
       <c r="A70" t="s">
         <v>31</v>
       </c>
@@ -3776,10 +3986,10 @@
         <v>0</v>
       </c>
       <c r="D70" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E70" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F70">
         <v>0.375</v>
@@ -3802,8 +4012,11 @@
       <c r="M70">
         <v>0.7723387723387725</v>
       </c>
-    </row>
-    <row r="71" spans="1:13">
+      <c r="N70">
+        <v>0.7723387723387725</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14">
       <c r="A71" t="s">
         <v>31</v>
       </c>
@@ -3814,10 +4027,10 @@
         <v>0</v>
       </c>
       <c r="D71" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E71" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F71">
         <v>0.5714285714285714</v>
@@ -3840,8 +4053,11 @@
       <c r="M71">
         <v>0.867909867909868</v>
       </c>
-    </row>
-    <row r="72" spans="1:13">
+      <c r="N71">
+        <v>0.867909867909868</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14">
       <c r="A72" t="s">
         <v>31</v>
       </c>
@@ -3852,10 +4068,10 @@
         <v>0</v>
       </c>
       <c r="D72" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E72" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F72">
         <v>0.5714285714285714</v>
@@ -3878,8 +4094,11 @@
       <c r="M72">
         <v>0.867909867909868</v>
       </c>
-    </row>
-    <row r="73" spans="1:13">
+      <c r="N72">
+        <v>0.867909867909868</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14">
       <c r="A73" t="s">
         <v>31</v>
       </c>
@@ -3890,10 +4109,10 @@
         <v>0</v>
       </c>
       <c r="D73" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E73" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F73">
         <v>0.4285714285714285</v>
@@ -3916,8 +4135,11 @@
       <c r="M73">
         <v>0.867909867909868</v>
       </c>
-    </row>
-    <row r="74" spans="1:13">
+      <c r="N73">
+        <v>0.867909867909868</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14">
       <c r="A74" t="s">
         <v>31</v>
       </c>
@@ -3928,10 +4150,10 @@
         <v>0</v>
       </c>
       <c r="D74" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E74" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F74">
         <v>0.4642857142857143</v>
@@ -3954,8 +4176,11 @@
       <c r="M74">
         <v>0.9284049284049285</v>
       </c>
-    </row>
-    <row r="75" spans="1:13">
+      <c r="N74">
+        <v>0.9284049284049285</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14">
       <c r="A75" t="s">
         <v>31</v>
       </c>
@@ -3966,10 +4191,10 @@
         <v>0</v>
       </c>
       <c r="D75" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E75" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F75">
         <v>0.4642857142857143</v>
@@ -3992,8 +4217,11 @@
       <c r="M75">
         <v>0.9284049284049285</v>
       </c>
-    </row>
-    <row r="76" spans="1:13">
+      <c r="N75">
+        <v>0.9284049284049285</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14">
       <c r="A76" t="s">
         <v>31</v>
       </c>
@@ -4004,10 +4232,10 @@
         <v>0</v>
       </c>
       <c r="D76" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E76" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F76">
         <v>0.4821428571428572</v>
@@ -4030,8 +4258,11 @@
       <c r="M76">
         <v>0.9550893550893552</v>
       </c>
-    </row>
-    <row r="77" spans="1:13">
+      <c r="N76">
+        <v>0.9550893550893552</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14">
       <c r="A77" t="s">
         <v>21</v>
       </c>
@@ -4042,10 +4273,10 @@
         <v>1</v>
       </c>
       <c r="D77" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E77" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F77">
         <v>0.8611111111111112</v>
@@ -4065,8 +4296,11 @@
       <c r="M77">
         <v>0.7812500000000002</v>
       </c>
-    </row>
-    <row r="78" spans="1:13">
+      <c r="N77">
+        <v>0.7812500000000002</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14">
       <c r="A78" t="s">
         <v>21</v>
       </c>
@@ -4077,10 +4311,10 @@
         <v>1</v>
       </c>
       <c r="D78" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E78" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F78">
         <v>0.8333333333333334</v>
@@ -4100,8 +4334,11 @@
       <c r="M78">
         <v>0.7812500000000002</v>
       </c>
-    </row>
-    <row r="79" spans="1:13">
+      <c r="N78">
+        <v>0.7812500000000002</v>
+      </c>
+    </row>
+    <row r="79" spans="1:14">
       <c r="A79" t="s">
         <v>21</v>
       </c>
@@ -4112,10 +4349,10 @@
         <v>1</v>
       </c>
       <c r="D79" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E79" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F79">
         <v>0.3333333333333333</v>
@@ -4135,8 +4372,11 @@
       <c r="M79">
         <v>0.7812500000000002</v>
       </c>
-    </row>
-    <row r="80" spans="1:13">
+      <c r="N79">
+        <v>0.7812500000000002</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14">
       <c r="A80" t="s">
         <v>21</v>
       </c>
@@ -4147,10 +4387,10 @@
         <v>1</v>
       </c>
       <c r="D80" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E80" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F80">
         <v>0.6944444444444444</v>
@@ -4170,8 +4410,11 @@
       <c r="M80">
         <v>0.7812500000000002</v>
       </c>
-    </row>
-    <row r="81" spans="1:13">
+      <c r="N80">
+        <v>0.7812500000000002</v>
+      </c>
+    </row>
+    <row r="81" spans="1:14">
       <c r="A81" t="s">
         <v>21</v>
       </c>
@@ -4182,10 +4425,10 @@
         <v>1</v>
       </c>
       <c r="D81" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E81" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F81">
         <v>0.2777777777777778</v>
@@ -4205,8 +4448,11 @@
       <c r="M81">
         <v>0.7812500000000002</v>
       </c>
-    </row>
-    <row r="82" spans="1:13">
+      <c r="N81">
+        <v>0.7812500000000002</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14">
       <c r="A82" t="s">
         <v>21</v>
       </c>
@@ -4217,10 +4463,10 @@
         <v>1</v>
       </c>
       <c r="D82" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E82" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F82">
         <v>0.1944444444444444</v>
@@ -4240,8 +4486,11 @@
       <c r="M82">
         <v>0.7812500000000002</v>
       </c>
-    </row>
-    <row r="83" spans="1:13">
+      <c r="N82">
+        <v>0.7812500000000002</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14">
       <c r="A83" t="s">
         <v>21</v>
       </c>
@@ -4252,10 +4501,10 @@
         <v>1</v>
       </c>
       <c r="D83" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E83" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F83">
         <v>0.6666666666666666</v>
@@ -4275,8 +4524,11 @@
       <c r="M83">
         <v>0.8437500000000003</v>
       </c>
-    </row>
-    <row r="84" spans="1:13">
+      <c r="N83">
+        <v>0.8437500000000003</v>
+      </c>
+    </row>
+    <row r="84" spans="1:14">
       <c r="A84" t="s">
         <v>21</v>
       </c>
@@ -4287,10 +4539,10 @@
         <v>1</v>
       </c>
       <c r="D84" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E84" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F84">
         <v>0.5555555555555556</v>
@@ -4310,8 +4562,11 @@
       <c r="M84">
         <v>0.8437500000000003</v>
       </c>
-    </row>
-    <row r="85" spans="1:13">
+      <c r="N84">
+        <v>0.8437500000000003</v>
+      </c>
+    </row>
+    <row r="85" spans="1:14">
       <c r="A85" t="s">
         <v>21</v>
       </c>
@@ -4322,10 +4577,10 @@
         <v>1</v>
       </c>
       <c r="D85" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E85" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F85">
         <v>0.6944444444444444</v>
@@ -4345,8 +4600,11 @@
       <c r="M85">
         <v>0.8437500000000003</v>
       </c>
-    </row>
-    <row r="86" spans="1:13">
+      <c r="N85">
+        <v>0.8437500000000003</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14">
       <c r="A86" t="s">
         <v>21</v>
       </c>
@@ -4357,10 +4615,10 @@
         <v>1</v>
       </c>
       <c r="D86" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E86" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F86">
         <v>0.6388888888888888</v>
@@ -4380,8 +4638,11 @@
       <c r="M86">
         <v>0.8437500000000003</v>
       </c>
-    </row>
-    <row r="87" spans="1:13">
+      <c r="N86">
+        <v>0.8437500000000003</v>
+      </c>
+    </row>
+    <row r="87" spans="1:14">
       <c r="A87" t="s">
         <v>21</v>
       </c>
@@ -4392,10 +4653,10 @@
         <v>1</v>
       </c>
       <c r="D87" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E87" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F87">
         <v>0.4722222222222222</v>
@@ -4415,8 +4676,11 @@
       <c r="M87">
         <v>0.8437500000000003</v>
       </c>
-    </row>
-    <row r="88" spans="1:13">
+      <c r="N87">
+        <v>0.8437500000000003</v>
+      </c>
+    </row>
+    <row r="88" spans="1:14">
       <c r="A88" t="s">
         <v>21</v>
       </c>
@@ -4427,10 +4691,10 @@
         <v>1</v>
       </c>
       <c r="D88" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E88" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F88">
         <v>0.5277777777777778</v>
@@ -4450,8 +4714,11 @@
       <c r="M88">
         <v>0.8437500000000003</v>
       </c>
-    </row>
-    <row r="89" spans="1:13">
+      <c r="N88">
+        <v>0.8437500000000003</v>
+      </c>
+    </row>
+    <row r="89" spans="1:14">
       <c r="A89" t="s">
         <v>21</v>
       </c>
@@ -4462,10 +4729,10 @@
         <v>1</v>
       </c>
       <c r="D89" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E89" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F89">
         <v>0.6666666666666666</v>
@@ -4485,8 +4752,11 @@
       <c r="M89">
         <v>0.8437500000000003</v>
       </c>
-    </row>
-    <row r="90" spans="1:13">
+      <c r="N89">
+        <v>0.8437500000000003</v>
+      </c>
+    </row>
+    <row r="90" spans="1:14">
       <c r="A90" t="s">
         <v>21</v>
       </c>
@@ -4497,10 +4767,10 @@
         <v>1</v>
       </c>
       <c r="D90" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E90" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F90">
         <v>0.3333333333333333</v>
@@ -4520,8 +4790,11 @@
       <c r="M90">
         <v>0.8437500000000003</v>
       </c>
-    </row>
-    <row r="91" spans="1:13">
+      <c r="N90">
+        <v>0.8437500000000003</v>
+      </c>
+    </row>
+    <row r="91" spans="1:14">
       <c r="A91" t="s">
         <v>21</v>
       </c>
@@ -4532,10 +4805,10 @@
         <v>1</v>
       </c>
       <c r="D91" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E91" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F91">
         <v>0.5</v>
@@ -4555,8 +4828,11 @@
       <c r="M91">
         <v>0.8437500000000003</v>
       </c>
-    </row>
-    <row r="92" spans="1:13">
+      <c r="N91">
+        <v>0.8437500000000003</v>
+      </c>
+    </row>
+    <row r="92" spans="1:14">
       <c r="A92" t="s">
         <v>23</v>
       </c>
@@ -4567,10 +4843,10 @@
         <v>1</v>
       </c>
       <c r="D92" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E92" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F92">
         <v>0.734375</v>
@@ -4590,8 +4866,11 @@
       <c r="M92">
         <v>0.8735795454545455</v>
       </c>
-    </row>
-    <row r="93" spans="1:13">
+      <c r="N92">
+        <v>0.8735795454545455</v>
+      </c>
+    </row>
+    <row r="93" spans="1:14">
       <c r="A93" t="s">
         <v>23</v>
       </c>
@@ -4602,10 +4881,10 @@
         <v>1</v>
       </c>
       <c r="D93" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E93" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F93">
         <v>0.609375</v>
@@ -4625,8 +4904,11 @@
       <c r="M93">
         <v>0.8735795454545455</v>
       </c>
-    </row>
-    <row r="94" spans="1:13">
+      <c r="N93">
+        <v>0.8735795454545455</v>
+      </c>
+    </row>
+    <row r="94" spans="1:14">
       <c r="A94" t="s">
         <v>23</v>
       </c>
@@ -4637,10 +4919,10 @@
         <v>1</v>
       </c>
       <c r="D94" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E94" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F94">
         <v>0.65625</v>
@@ -4660,8 +4942,11 @@
       <c r="M94">
         <v>0.8735795454545455</v>
       </c>
-    </row>
-    <row r="95" spans="1:13">
+      <c r="N94">
+        <v>0.8735795454545455</v>
+      </c>
+    </row>
+    <row r="95" spans="1:14">
       <c r="A95" t="s">
         <v>23</v>
       </c>
@@ -4672,10 +4957,10 @@
         <v>1</v>
       </c>
       <c r="D95" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E95" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F95">
         <v>0.59375</v>
@@ -4695,8 +4980,11 @@
       <c r="M95">
         <v>0.8735795454545455</v>
       </c>
-    </row>
-    <row r="96" spans="1:13">
+      <c r="N95">
+        <v>0.8735795454545455</v>
+      </c>
+    </row>
+    <row r="96" spans="1:14">
       <c r="A96" t="s">
         <v>23</v>
       </c>
@@ -4707,10 +4995,10 @@
         <v>1</v>
       </c>
       <c r="D96" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E96" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F96">
         <v>0.390625</v>
@@ -4730,8 +5018,11 @@
       <c r="M96">
         <v>0.8735795454545455</v>
       </c>
-    </row>
-    <row r="97" spans="1:13">
+      <c r="N96">
+        <v>0.8735795454545455</v>
+      </c>
+    </row>
+    <row r="97" spans="1:14">
       <c r="A97" t="s">
         <v>23</v>
       </c>
@@ -4742,10 +5033,10 @@
         <v>1</v>
       </c>
       <c r="D97" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E97" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F97">
         <v>0.390625</v>
@@ -4765,8 +5056,11 @@
       <c r="M97">
         <v>0.8735795454545455</v>
       </c>
-    </row>
-    <row r="98" spans="1:13">
+      <c r="N97">
+        <v>0.8735795454545455</v>
+      </c>
+    </row>
+    <row r="98" spans="1:14">
       <c r="A98" t="s">
         <v>23</v>
       </c>
@@ -4777,10 +5071,10 @@
         <v>1</v>
       </c>
       <c r="D98" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E98" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F98">
         <v>0.4375</v>
@@ -4800,8 +5094,11 @@
       <c r="M98">
         <v>0.8735795454545455</v>
       </c>
-    </row>
-    <row r="99" spans="1:13">
+      <c r="N98">
+        <v>0.8735795454545455</v>
+      </c>
+    </row>
+    <row r="99" spans="1:14">
       <c r="A99" t="s">
         <v>23</v>
       </c>
@@ -4812,10 +5109,10 @@
         <v>1</v>
       </c>
       <c r="D99" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E99" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F99">
         <v>0.421875</v>
@@ -4835,8 +5132,11 @@
       <c r="M99">
         <v>0.8735795454545455</v>
       </c>
-    </row>
-    <row r="100" spans="1:13">
+      <c r="N99">
+        <v>0.8735795454545455</v>
+      </c>
+    </row>
+    <row r="100" spans="1:14">
       <c r="A100" t="s">
         <v>23</v>
       </c>
@@ -4847,10 +5147,10 @@
         <v>1</v>
       </c>
       <c r="D100" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E100" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F100">
         <v>0.34375</v>
@@ -4870,8 +5170,11 @@
       <c r="M100">
         <v>0.8735795454545455</v>
       </c>
-    </row>
-    <row r="101" spans="1:13">
+      <c r="N100">
+        <v>0.8735795454545455</v>
+      </c>
+    </row>
+    <row r="101" spans="1:14">
       <c r="A101" t="s">
         <v>23</v>
       </c>
@@ -4882,10 +5185,10 @@
         <v>1</v>
       </c>
       <c r="D101" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E101" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F101">
         <v>0.65625</v>
@@ -4905,8 +5208,11 @@
       <c r="M101">
         <v>0.8735795454545455</v>
       </c>
-    </row>
-    <row r="102" spans="1:13">
+      <c r="N101">
+        <v>0.8735795454545455</v>
+      </c>
+    </row>
+    <row r="102" spans="1:14">
       <c r="A102" t="s">
         <v>23</v>
       </c>
@@ -4917,10 +5223,10 @@
         <v>1</v>
       </c>
       <c r="D102" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E102" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F102">
         <v>0.625</v>
@@ -4940,8 +5246,11 @@
       <c r="M102">
         <v>0.8735795454545455</v>
       </c>
-    </row>
-    <row r="103" spans="1:13">
+      <c r="N102">
+        <v>0.8735795454545455</v>
+      </c>
+    </row>
+    <row r="103" spans="1:14">
       <c r="A103" t="s">
         <v>23</v>
       </c>
@@ -4952,10 +5261,10 @@
         <v>1</v>
       </c>
       <c r="D103" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E103" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F103">
         <v>0.578125</v>
@@ -4975,8 +5284,11 @@
       <c r="M103">
         <v>0.9040178571428572</v>
       </c>
-    </row>
-    <row r="104" spans="1:13">
+      <c r="N103">
+        <v>0.9040178571428572</v>
+      </c>
+    </row>
+    <row r="104" spans="1:14">
       <c r="A104" t="s">
         <v>23</v>
       </c>
@@ -4987,10 +5299,10 @@
         <v>1</v>
       </c>
       <c r="D104" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E104" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F104">
         <v>0.515625</v>
@@ -5010,8 +5322,11 @@
       <c r="M104">
         <v>0.9040178571428572</v>
       </c>
-    </row>
-    <row r="105" spans="1:13">
+      <c r="N104">
+        <v>0.9040178571428572</v>
+      </c>
+    </row>
+    <row r="105" spans="1:14">
       <c r="A105" t="s">
         <v>23</v>
       </c>
@@ -5022,10 +5337,10 @@
         <v>1</v>
       </c>
       <c r="D105" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E105" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F105">
         <v>0.453125</v>
@@ -5045,8 +5360,11 @@
       <c r="M105">
         <v>0.9040178571428572</v>
       </c>
-    </row>
-    <row r="106" spans="1:13">
+      <c r="N105">
+        <v>0.9040178571428572</v>
+      </c>
+    </row>
+    <row r="106" spans="1:14">
       <c r="A106" t="s">
         <v>23</v>
       </c>
@@ -5057,10 +5375,10 @@
         <v>1</v>
       </c>
       <c r="D106" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E106" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F106">
         <v>0.453125</v>
@@ -5080,8 +5398,11 @@
       <c r="M106">
         <v>0.9453124999999998</v>
       </c>
-    </row>
-    <row r="107" spans="1:13">
+      <c r="N106">
+        <v>0.9453124999999998</v>
+      </c>
+    </row>
+    <row r="107" spans="1:14">
       <c r="A107" t="s">
         <v>33</v>
       </c>
@@ -5092,10 +5413,10 @@
         <v>0</v>
       </c>
       <c r="D107" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E107" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F107">
         <v>0.8333333333333334</v>
@@ -5118,8 +5439,11 @@
       <c r="M107">
         <v>0.6393606393606394</v>
       </c>
-    </row>
-    <row r="108" spans="1:13">
+      <c r="N107">
+        <v>0.6393606393606394</v>
+      </c>
+    </row>
+    <row r="108" spans="1:14">
       <c r="A108" t="s">
         <v>33</v>
       </c>
@@ -5130,10 +5454,10 @@
         <v>0</v>
       </c>
       <c r="D108" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E108" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F108">
         <v>0.7083333333333334</v>
@@ -5156,8 +5480,11 @@
       <c r="M108">
         <v>0.8471528471528473</v>
       </c>
-    </row>
-    <row r="109" spans="1:13">
+      <c r="N108">
+        <v>0.8471528471528473</v>
+      </c>
+    </row>
+    <row r="109" spans="1:14">
       <c r="A109" t="s">
         <v>33</v>
       </c>
@@ -5168,10 +5495,10 @@
         <v>0</v>
       </c>
       <c r="D109" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E109" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F109">
         <v>0.6875</v>
@@ -5194,8 +5521,11 @@
       <c r="M109">
         <v>0.8471528471528473</v>
       </c>
-    </row>
-    <row r="110" spans="1:13">
+      <c r="N109">
+        <v>0.8471528471528473</v>
+      </c>
+    </row>
+    <row r="110" spans="1:14">
       <c r="A110" t="s">
         <v>33</v>
       </c>
@@ -5206,10 +5536,10 @@
         <v>0</v>
       </c>
       <c r="D110" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E110" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F110">
         <v>0.3125</v>
@@ -5232,8 +5562,11 @@
       <c r="M110">
         <v>0.8471528471528473</v>
       </c>
-    </row>
-    <row r="111" spans="1:13">
+      <c r="N110">
+        <v>0.8471528471528473</v>
+      </c>
+    </row>
+    <row r="111" spans="1:14">
       <c r="A111" t="s">
         <v>33</v>
       </c>
@@ -5244,10 +5577,10 @@
         <v>0</v>
       </c>
       <c r="D111" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E111" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F111">
         <v>0.3125</v>
@@ -5270,8 +5603,11 @@
       <c r="M111">
         <v>0.8471528471528473</v>
       </c>
-    </row>
-    <row r="112" spans="1:13">
+      <c r="N111">
+        <v>0.8471528471528473</v>
+      </c>
+    </row>
+    <row r="112" spans="1:14">
       <c r="A112" t="s">
         <v>33</v>
       </c>
@@ -5282,10 +5618,10 @@
         <v>0</v>
       </c>
       <c r="D112" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E112" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F112">
         <v>0.625</v>
@@ -5308,8 +5644,11 @@
       <c r="M112">
         <v>0.9546009546009547</v>
       </c>
-    </row>
-    <row r="113" spans="1:13">
+      <c r="N112">
+        <v>0.9546009546009547</v>
+      </c>
+    </row>
+    <row r="113" spans="1:14">
       <c r="A113" t="s">
         <v>33</v>
       </c>
@@ -5320,10 +5659,10 @@
         <v>0</v>
       </c>
       <c r="D113" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E113" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F113">
         <v>0.3958333333333333</v>
@@ -5346,8 +5685,11 @@
       <c r="M113">
         <v>0.9546009546009547</v>
       </c>
-    </row>
-    <row r="114" spans="1:13">
+      <c r="N113">
+        <v>0.9546009546009547</v>
+      </c>
+    </row>
+    <row r="114" spans="1:14">
       <c r="A114" t="s">
         <v>33</v>
       </c>
@@ -5358,10 +5700,10 @@
         <v>0</v>
       </c>
       <c r="D114" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E114" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F114">
         <v>0.6041666666666666</v>
@@ -5384,8 +5726,11 @@
       <c r="M114">
         <v>0.9546009546009547</v>
       </c>
-    </row>
-    <row r="115" spans="1:13">
+      <c r="N114">
+        <v>0.9546009546009547</v>
+      </c>
+    </row>
+    <row r="115" spans="1:14">
       <c r="A115" t="s">
         <v>33</v>
       </c>
@@ -5396,10 +5741,10 @@
         <v>0</v>
       </c>
       <c r="D115" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E115" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F115">
         <v>0.3958333333333333</v>
@@ -5422,8 +5767,11 @@
       <c r="M115">
         <v>0.9546009546009547</v>
       </c>
-    </row>
-    <row r="116" spans="1:13">
+      <c r="N115">
+        <v>0.9546009546009547</v>
+      </c>
+    </row>
+    <row r="116" spans="1:14">
       <c r="A116" t="s">
         <v>33</v>
       </c>
@@ -5434,10 +5782,10 @@
         <v>0</v>
       </c>
       <c r="D116" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E116" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F116">
         <v>0.4166666666666667</v>
@@ -5460,8 +5808,11 @@
       <c r="M116">
         <v>0.993006993006993</v>
       </c>
-    </row>
-    <row r="117" spans="1:13">
+      <c r="N116">
+        <v>0.993006993006993</v>
+      </c>
+    </row>
+    <row r="117" spans="1:14">
       <c r="A117" t="s">
         <v>33</v>
       </c>
@@ -5472,10 +5823,10 @@
         <v>0</v>
       </c>
       <c r="D117" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E117" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F117">
         <v>0.5416666666666666</v>
@@ -5498,8 +5849,11 @@
       <c r="M117">
         <v>1</v>
       </c>
-    </row>
-    <row r="118" spans="1:13">
+      <c r="N117">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118" spans="1:14">
       <c r="A118" t="s">
         <v>33</v>
       </c>
@@ -5510,10 +5864,10 @@
         <v>0</v>
       </c>
       <c r="D118" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E118" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F118">
         <v>0.5416666666666666</v>
@@ -5536,8 +5890,11 @@
       <c r="M118">
         <v>1</v>
       </c>
-    </row>
-    <row r="119" spans="1:13">
+      <c r="N118">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119" spans="1:14">
       <c r="A119" t="s">
         <v>33</v>
       </c>
@@ -5548,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="D119" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E119" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F119">
         <v>0.4791666666666667</v>
@@ -5574,8 +5931,11 @@
       <c r="M119">
         <v>1</v>
       </c>
-    </row>
-    <row r="120" spans="1:13">
+      <c r="N119">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120" spans="1:14">
       <c r="A120" t="s">
         <v>33</v>
       </c>
@@ -5586,10 +5946,10 @@
         <v>0</v>
       </c>
       <c r="D120" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E120" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F120">
         <v>0.4791666666666667</v>
@@ -5612,8 +5972,11 @@
       <c r="M120">
         <v>1</v>
       </c>
-    </row>
-    <row r="121" spans="1:13">
+      <c r="N120">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121" spans="1:14">
       <c r="A121" t="s">
         <v>33</v>
       </c>
@@ -5624,10 +5987,10 @@
         <v>0</v>
       </c>
       <c r="D121" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E121" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F121">
         <v>0.5</v>
@@ -5648,6 +6011,9 @@
         <v>8</v>
       </c>
       <c r="M121">
+        <v>1</v>
+      </c>
+      <c r="N121">
         <v>1</v>
       </c>
     </row>
@@ -5669,21 +6035,21 @@
         <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>37</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -5694,13 +6060,13 @@
         <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -5711,13 +6077,13 @@
         <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C4">
         <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E4">
         <v>2</v>
@@ -5728,13 +6094,13 @@
         <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C5">
         <v>2</v>
       </c>
       <c r="D5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E5">
         <v>3</v>
@@ -5745,13 +6111,13 @@
         <v>27</v>
       </c>
       <c r="B6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C6">
         <v>3</v>
       </c>
       <c r="D6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -5762,13 +6128,13 @@
         <v>27</v>
       </c>
       <c r="B7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C7">
         <v>3</v>
       </c>
       <c r="D7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E7">
         <v>2</v>
@@ -5779,13 +6145,13 @@
         <v>27</v>
       </c>
       <c r="B8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C8">
         <v>3</v>
       </c>
       <c r="D8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E8">
         <v>3</v>
@@ -5796,13 +6162,13 @@
         <v>27</v>
       </c>
       <c r="B9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C9">
         <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E9">
         <v>4</v>
@@ -5813,13 +6179,13 @@
         <v>27</v>
       </c>
       <c r="B10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C10">
         <v>3</v>
       </c>
       <c r="D10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E10">
         <v>5</v>
@@ -5830,13 +6196,13 @@
         <v>27</v>
       </c>
       <c r="B11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C11">
         <v>3</v>
       </c>
       <c r="D11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E11">
         <v>6</v>
@@ -5847,13 +6213,13 @@
         <v>29</v>
       </c>
       <c r="B12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C12">
         <v>4</v>
       </c>
       <c r="D12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -5864,13 +6230,13 @@
         <v>33</v>
       </c>
       <c r="B13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C13">
         <v>5</v>
       </c>
       <c r="D13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -5881,13 +6247,13 @@
         <v>35</v>
       </c>
       <c r="B14" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C14">
         <v>6</v>
       </c>
       <c r="D14" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -5905,24 +6271,24 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -5937,596 +6303,596 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4" t="s">
         <v>78</v>
-      </c>
-      <c r="B4" t="s">
-        <v>79</v>
-      </c>
-      <c r="C4" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B10" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B11" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C11" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B12" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C13" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C14" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B15" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C15" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B16" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B17" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B18" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B19" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C19" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B20" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C20" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B21" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C21" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B22" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C22" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B23" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C23" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B24" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C24" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B25" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C25" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B26" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C26" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C27" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B28" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C28" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B29" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C29" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B30" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C30" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B31" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C31" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B32" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C32" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B33" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C33" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B34" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C34" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B35" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C35" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B36" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C36" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B37" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C37" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B38" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C38" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B39" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C39" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C40" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B41" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C41" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B42" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C42" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B43" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C43" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B44" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C44" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B45" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C45" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B46" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C46" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B47" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C47" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B48" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C48" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B49" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C49" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B50" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C50" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B51" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C51" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B52" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C52" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B53" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C53" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B54" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C54" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>

</xml_diff>